<commit_message>
Completa ago-sep 2026 con el extracto de convenio marco de Datos Abiertos
- Recupera OC SE/CC sin código en ago y sep 2026 (+490 OC, +1,1% del monto),
  principalmente Pasajes, Beneficios y Seguro.
- Tipo de producto con correspondencias de ago y sep 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/administracion-y-entrega-de-beneficios/ago-2026.xlsx
+++ b/docs/oc-mensuales/administracion-y-entrega-de-beneficios/ago-2026.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M320"/>
+  <dimension ref="A1:M322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10589,7 +10589,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>4777-668-CM26</t>
+          <t>4305-108-CM26</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -10609,22 +10609,22 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>69.200.800-6</t>
+          <t>61.943.400-5</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LA UNION</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Magallanes</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10648,7 +10648,7 @@
         </is>
       </c>
       <c r="M157" s="2" t="n">
-        <v>749.0599999999999</v>
+        <v>7926.78</v>
       </c>
     </row>
     <row r="158">
@@ -10719,7 +10719,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>4305-108-CM26</t>
+          <t>4777-668-CM26</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -10739,22 +10739,22 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>61.943.400-5</t>
+          <t>69.200.800-6</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>I MUNICIPALIDAD DE LA UNION</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Magallanes</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10778,7 +10778,7 @@
         </is>
       </c>
       <c r="M159" s="2" t="n">
-        <v>7926.78</v>
+        <v>749.0599999999999</v>
       </c>
     </row>
     <row r="160">
@@ -10849,7 +10849,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>1078177-747-CM26</t>
+          <t>1078177-745-CM26</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -10908,13 +10908,13 @@
         </is>
       </c>
       <c r="M161" s="2" t="n">
-        <v>19357.46</v>
+        <v>7137.91</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>1078177-745-CM26</t>
+          <t>1078177-747-CM26</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -10973,7 +10973,7 @@
         </is>
       </c>
       <c r="M162" s="2" t="n">
-        <v>7137.91</v>
+        <v>19357.46</v>
       </c>
     </row>
     <row r="163">
@@ -12929,7 +12929,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>707416-68-CM26</t>
+          <t>1080286-352-CM26</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -12954,27 +12954,27 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>70.574.900-0</t>
+          <t>61.978.700-5</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>FUNDACION EDUCACIONAL PARA EL DESAROLLO INTEGRAL DE LA NIÑEZ</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Atacama</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12988,13 +12988,13 @@
         </is>
       </c>
       <c r="M193" s="2" t="n">
-        <v>5259.83</v>
+        <v>325.99</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>1080286-352-CM26</t>
+          <t>1294154-2-CM26</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -13014,17 +13014,17 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>61.978.700-5</t>
+          <t>65.034.169-4</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>Consejo Resolutivo de Asignaciones Parlamentaria</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -13034,12 +13034,12 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -13053,7 +13053,7 @@
         </is>
       </c>
       <c r="M194" s="2" t="n">
-        <v>325.99</v>
+        <v>11866.21</v>
       </c>
     </row>
     <row r="195">
@@ -13124,7 +13124,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>1294154-2-CM26</t>
+          <t>707416-68-CM26</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -13144,22 +13144,22 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>65.034.169-4</t>
+          <t>70.574.900-0</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Consejo Resolutivo de Asignaciones Parlamentaria</t>
+          <t>FUNDACION EDUCACIONAL PARA EL DESAROLLO INTEGRAL DE LA NIÑEZ</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -13183,7 +13183,7 @@
         </is>
       </c>
       <c r="M196" s="2" t="n">
-        <v>11866.21</v>
+        <v>5259.83</v>
       </c>
     </row>
     <row r="197">
@@ -13319,7 +13319,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>617807-4713-CM26</t>
+          <t>683-32-CM26</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -13339,22 +13339,22 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>61.602.036-6</t>
+          <t>61.402.008-3</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>SERV NAC SALUD HOSPITAL DE LOS ANDES</t>
+          <t>MINISTERIO DE BIENES NACIONALES</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Magallanes</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13378,13 +13378,13 @@
         </is>
       </c>
       <c r="M199" s="2" t="n">
-        <v>1064.92</v>
+        <v>814.99</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>683-32-CM26</t>
+          <t>617807-4713-CM26</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -13404,22 +13404,22 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>61.402.008-3</t>
+          <t>61.602.036-6</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>MINISTERIO DE BIENES NACIONALES</t>
+          <t>SERV NAC SALUD HOSPITAL DE LOS ANDES</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Magallanes</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13443,7 +13443,7 @@
         </is>
       </c>
       <c r="M200" s="2" t="n">
-        <v>814.99</v>
+        <v>1064.92</v>
       </c>
     </row>
     <row r="201">
@@ -15464,7 +15464,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>3474-475-CM26</t>
+          <t>889473-1465-CM26</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -15489,17 +15489,17 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>61.979.960-7</t>
+          <t>61.980.530-5</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>UNIVERSIDAD DE O'HIGGINS</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15523,13 +15523,13 @@
         </is>
       </c>
       <c r="M232" s="2" t="n">
-        <v>2038.66</v>
+        <v>11263.19</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>1079694-291-CM26</t>
+          <t>2107-1711-CM26</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -15554,27 +15554,27 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>60.505.523-0</t>
+          <t>61.602.148-6</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE SANTA CRUZ</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15588,13 +15588,13 @@
         </is>
       </c>
       <c r="M233" s="2" t="n">
-        <v>38736.49</v>
+        <v>56852.97</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>3453-417-CM26</t>
+          <t>1383-263-CM26</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -15614,22 +15614,22 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>61.979.960-7</t>
+          <t>61.602.242-3</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>HOSPITAL VILCUN</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -15653,13 +15653,13 @@
         </is>
       </c>
       <c r="M234" s="2" t="n">
-        <v>26846.5</v>
+        <v>10279.54</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2107-1711-CM26</t>
+          <t>1079694-291-CM26</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -15684,27 +15684,27 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>61.602.148-6</t>
+          <t>60.505.523-0</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE SANTA CRUZ</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15718,13 +15718,13 @@
         </is>
       </c>
       <c r="M235" s="2" t="n">
-        <v>56852.97</v>
+        <v>38736.49</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>889473-1465-CM26</t>
+          <t>3474-475-CM26</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -15749,17 +15749,17 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>61.980.530-5</t>
+          <t>61.979.960-7</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>UNIVERSIDAD DE O'HIGGINS</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15783,13 +15783,13 @@
         </is>
       </c>
       <c r="M236" s="2" t="n">
-        <v>11263.19</v>
+        <v>2038.66</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>1383-263-CM26</t>
+          <t>3453-417-CM26</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -15809,22 +15809,22 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>61.602.242-3</t>
+          <t>61.979.960-7</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>HOSPITAL VILCUN</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15848,13 +15848,13 @@
         </is>
       </c>
       <c r="M237" s="2" t="n">
-        <v>10279.54</v>
+        <v>26846.5</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>1622-1104-CM26</t>
+          <t>1057438-237-CM26</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -15879,27 +15879,27 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>61.602.141-9</t>
+          <t>61.606.401-0</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE SAN VICENTE DE TAGUA TAGUA</t>
+          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL VICUNA</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15913,13 +15913,13 @@
         </is>
       </c>
       <c r="M238" s="2" t="n">
-        <v>25146.51</v>
+        <v>14477.85</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>1057534-1092-CM26</t>
+          <t>1622-1104-CM26</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -15944,17 +15944,17 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>61.607.602-7</t>
+          <t>61.602.141-9</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD OSORNO HOSPITAL PURRANQUE</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE SAN VICENTE DE TAGUA TAGUA</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>Los Lagos</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15978,13 +15978,13 @@
         </is>
       </c>
       <c r="M239" s="2" t="n">
-        <v>24053.18</v>
+        <v>25146.51</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2776-543-CM26</t>
+          <t>1057534-1092-CM26</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -16009,17 +16009,17 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>69.081.200-2</t>
+          <t>61.607.602-7</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE RENGO</t>
+          <t>SERVICIO DE SALUD OSORNO HOSPITAL PURRANQUE</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -16043,13 +16043,13 @@
         </is>
       </c>
       <c r="M240" s="2" t="n">
-        <v>13119.92</v>
+        <v>24053.18</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>1375760-65-CM26</t>
+          <t>2776-543-CM26</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -16069,32 +16069,32 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>61.981.310-3</t>
+          <t>69.081.200-2</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>SERVICIO LOCAL DE EDUCACIÓN PÚBLICA VALLE CACHAPOAL</t>
+          <t>I MUNICIPALIDAD DE RENGO</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -16108,13 +16108,13 @@
         </is>
       </c>
       <c r="M241" s="2" t="n">
-        <v>1790.23</v>
+        <v>13119.92</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>3544-205-CM26</t>
+          <t>1375760-65-CM26</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -16134,32 +16134,32 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>61.101.062-1</t>
+          <t>61.981.310-3</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>SERVICIO LOCAL DE EDUCACIÓN PÚBLICA VALLE CACHAPOAL</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -16173,13 +16173,13 @@
         </is>
       </c>
       <c r="M242" s="2" t="n">
-        <v>470.13</v>
+        <v>1790.23</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2378-291-CM26</t>
+          <t>3544-205-CM26</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -16199,32 +16199,32 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>69.070.700-4</t>
+          <t>61.101.062-1</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LA FLORIDA</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16238,13 +16238,13 @@
         </is>
       </c>
       <c r="M243" s="2" t="n">
-        <v>3553.31</v>
+        <v>470.13</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>3544-201-CM26</t>
+          <t>2378-291-CM26</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -16264,32 +16264,32 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>61.101.062-1</t>
+          <t>69.070.700-4</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>I MUNICIPALIDAD DE LA FLORIDA</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16303,13 +16303,13 @@
         </is>
       </c>
       <c r="M244" s="2" t="n">
-        <v>1639.99</v>
+        <v>3553.31</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>5701-112-CM26</t>
+          <t>3544-201-CM26</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -16329,22 +16329,22 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>60.505.000-K</t>
+          <t>61.101.062-1</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -16368,13 +16368,13 @@
         </is>
       </c>
       <c r="M245" s="2" t="n">
-        <v>15809.39</v>
+        <v>1639.99</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>1057438-237-CM26</t>
+          <t>5701-112-CM26</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -16394,32 +16394,32 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>61.606.401-0</t>
+          <t>60.505.000-K</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL VICUNA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>Coquimbo</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16433,18 +16433,18 @@
         </is>
       </c>
       <c r="M246" s="2" t="n">
-        <v>14477.85</v>
+        <v>15809.39</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>1624-196-CM26</t>
+          <t>1627-1161-SE26</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2239-1-LR26</t>
+          <t>2239-2-LR21</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -16454,22 +16454,22 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>61.602.147-8</t>
+          <t>61.602.145-1</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE NANCAGUA</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE SAN FERNANDO</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -16498,13 +16498,13 @@
         </is>
       </c>
       <c r="M247" s="2" t="n">
-        <v>9916.34</v>
+        <v>84659.45</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>3474-481-CM26</t>
+          <t>1624-196-CM26</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -16529,17 +16529,17 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>61.979.960-7</t>
+          <t>61.602.147-8</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE NANCAGUA</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -16563,13 +16563,13 @@
         </is>
       </c>
       <c r="M248" s="2" t="n">
-        <v>376.33</v>
+        <v>9916.34</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>1628-247-CM26</t>
+          <t>3474-481-CM26</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -16594,17 +16594,17 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>61.602.132-k</t>
+          <t>61.979.960-7</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE GRANEROS</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -16628,13 +16628,13 @@
         </is>
       </c>
       <c r="M249" s="2" t="n">
-        <v>16457.65</v>
+        <v>376.33</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>1490160-92-CM26</t>
+          <t>1628-247-CM26</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -16654,22 +16654,22 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>61.981.260-3</t>
+          <t>61.602.132-k</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>SERVICIO LOCAL DE EDUCACIÓN PÚBLICA LOS PARQUES</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE GRANEROS</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16693,13 +16693,13 @@
         </is>
       </c>
       <c r="M250" s="2" t="n">
-        <v>4257.05</v>
+        <v>16457.65</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2205-123-CM26</t>
+          <t>1490160-92-CM26</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -16719,22 +16719,22 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>61.602.143-5</t>
+          <t>61.981.260-3</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE PICHIDEGUA</t>
+          <t>SERVICIO LOCAL DE EDUCACIÓN PÚBLICA LOS PARQUES</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -16758,13 +16758,13 @@
         </is>
       </c>
       <c r="M251" s="2" t="n">
-        <v>6397.64</v>
+        <v>4257.05</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>1043046-93-CM26</t>
+          <t>2205-123-CM26</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -16784,22 +16784,22 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>62.000.450-2</t>
+          <t>61.602.143-5</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>DELEGACIÓN PRESIDENCIAL REGIONAL DE ÑUBLE</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE PICHIDEGUA</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -16823,13 +16823,13 @@
         </is>
       </c>
       <c r="M252" s="2" t="n">
-        <v>3244.81</v>
+        <v>6397.64</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2412-514-CM26</t>
+          <t>1043046-93-CM26</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -16849,22 +16849,22 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>69.254.100-6</t>
+          <t>62.000.450-2</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LO PRADO</t>
+          <t>DELEGACIÓN PRESIDENCIAL REGIONAL DE ÑUBLE</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -16888,13 +16888,13 @@
         </is>
       </c>
       <c r="M253" s="2" t="n">
-        <v>281.43</v>
+        <v>3244.81</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>1057496-1506-CM26</t>
+          <t>2412-514-CM26</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -16919,12 +16919,12 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>61.608.105-5</t>
+          <t>69.254.100-6</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD SUR HOSPITAL SAN LUIS</t>
+          <t>I MUNICIPALIDAD DE LO PRADO</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -16953,13 +16953,13 @@
         </is>
       </c>
       <c r="M254" s="2" t="n">
-        <v>5544.83</v>
+        <v>281.43</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>1552-424-CM26</t>
+          <t>1057496-1506-CM26</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -16984,17 +16984,17 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>61.606.300-6</t>
+          <t>61.608.105-5</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD ATACAMA</t>
+          <t>SERVICIO DE SALUD SUR HOSPITAL SAN LUIS</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>Atacama</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -17018,13 +17018,13 @@
         </is>
       </c>
       <c r="M255" s="2" t="n">
-        <v>38401.19</v>
+        <v>5544.83</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>1705-549-CM26</t>
+          <t>1552-424-CM26</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -17049,17 +17049,17 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>61.606.603-k</t>
+          <t>61.606.300-6</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>HOSPITAL ADRIANA COUSINO DE QUINTERO</t>
+          <t>SERVICIO DE SALUD ATACAMA</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -17083,13 +17083,13 @@
         </is>
       </c>
       <c r="M256" s="2" t="n">
-        <v>25235.07</v>
+        <v>38401.19</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>1070329-235-CM26</t>
+          <t>1705-549-CM26</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -17114,17 +17114,17 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>61.980.370-1</t>
+          <t>61.606.603-k</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>CESFAM LIRQUEN</t>
+          <t>HOSPITAL ADRIANA COUSINO DE QUINTERO</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -17148,13 +17148,13 @@
         </is>
       </c>
       <c r="M257" s="2" t="n">
-        <v>15141.93</v>
+        <v>25235.07</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2102-735-CM26</t>
+          <t>1070329-235-CM26</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -17179,12 +17179,12 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>61.602.212-1</t>
+          <t>61.980.370-1</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>SERVICIO NACIONAL DE SALUD HOSPITAL DE LEBU</t>
+          <t>CESFAM LIRQUEN</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -17213,13 +17213,13 @@
         </is>
       </c>
       <c r="M258" s="2" t="n">
-        <v>50557.56</v>
+        <v>15141.93</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>1391-1676-CM26</t>
+          <t>2102-735-CM26</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -17244,17 +17244,17 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>61.004.051-9</t>
+          <t>61.602.212-1</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
+          <t>SERVICIO NACIONAL DE SALUD HOSPITAL DE LEBU</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -17278,13 +17278,13 @@
         </is>
       </c>
       <c r="M259" s="2" t="n">
-        <v>3489.02</v>
+        <v>50557.56</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2170-870-CM26</t>
+          <t>1391-1676-CM26</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -17309,17 +17309,17 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>61.606.606-4</t>
+          <t>61.004.051-9</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>HOSPITAL DE LA FAMILIA Y LA COMUNIDAD SANTO TOMAS DE LIMACHE</t>
+          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17343,13 +17343,13 @@
         </is>
       </c>
       <c r="M260" s="2" t="n">
-        <v>6113.24</v>
+        <v>3489.02</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2170-869-CM26</t>
+          <t>2170-870-CM26</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -17408,13 +17408,13 @@
         </is>
       </c>
       <c r="M261" s="2" t="n">
-        <v>23878.25</v>
+        <v>6113.24</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2080-8552-CM26</t>
+          <t>2170-869-CM26</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -17439,17 +17439,17 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>61.602.138-9</t>
+          <t>61.606.606-4</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL LIBERTADOR B O'HIGGINS HOSPITAL REG RANCAGUA</t>
+          <t>HOSPITAL DE LA FAMILIA Y LA COMUNIDAD SANTO TOMAS DE LIMACHE</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -17473,13 +17473,13 @@
         </is>
       </c>
       <c r="M262" s="2" t="n">
-        <v>12617.69</v>
+        <v>23878.25</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>1079713-493-CM26</t>
+          <t>2080-8552-CM26</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -17494,7 +17494,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -17504,17 +17504,17 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>53.322.604-3</t>
+          <t>61.602.138-9</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SERVICIO DE SALUD DEL LIBERTADOR B O'HIGGINS HOSPITAL REG RANCAGUA</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -17538,13 +17538,13 @@
         </is>
       </c>
       <c r="M263" s="2" t="n">
-        <v>75555.67</v>
+        <v>12617.69</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>2186-754-CM26</t>
+          <t>1079713-493-CM26</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -17569,17 +17569,17 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>61.606.607-2</t>
+          <t>53.322.604-3</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>HOSPITAL GERIATRICO LA PAZ DE LA TARDE</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -17603,13 +17603,13 @@
         </is>
       </c>
       <c r="M264" s="2" t="n">
-        <v>15872.37</v>
+        <v>75555.67</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>3553-383-CM26</t>
+          <t>2186-754-CM26</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -17629,22 +17629,22 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>61.402.000-8</t>
+          <t>61.606.607-2</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>MINISTERIO DE BIENES NACIONALES</t>
+          <t>HOSPITAL GERIATRICO LA PAZ DE LA TARDE</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -17668,13 +17668,13 @@
         </is>
       </c>
       <c r="M265" s="2" t="n">
-        <v>26738.86</v>
+        <v>15872.37</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>1620-202-CM26</t>
+          <t>3553-383-CM26</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -17694,22 +17694,22 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>61.602.146-k</t>
+          <t>61.402.000-8</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE CHIMBARONGO</t>
+          <t>MINISTERIO DE BIENES NACIONALES</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -17733,13 +17733,13 @@
         </is>
       </c>
       <c r="M266" s="2" t="n">
-        <v>17421.51</v>
+        <v>26738.86</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>3515-387-CM26</t>
+          <t>1620-202-CM26</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -17759,22 +17759,22 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>69.060.300-4</t>
+          <t>61.602.146-k</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LA CALERA</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE CHIMBARONGO</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -17798,13 +17798,13 @@
         </is>
       </c>
       <c r="M267" s="2" t="n">
-        <v>1088.83</v>
+        <v>17421.51</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>972135-11-CM26</t>
+          <t>3515-387-CM26</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -17824,22 +17824,22 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>69.150.400-k</t>
+          <t>69.060.300-4</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE CONCEPCION</t>
+          <t>I MUNICIPALIDAD DE LA CALERA</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -17863,13 +17863,13 @@
         </is>
       </c>
       <c r="M268" s="2" t="n">
-        <v>15787.98</v>
+        <v>1088.83</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>682-31-CM26</t>
+          <t>972135-11-CM26</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -17894,17 +17894,17 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>61.802.014-2</t>
+          <t>69.150.400-k</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>MINISTERIO DE BIENES NACIONALES</t>
+          <t>I MUNICIPALIDAD DE CONCEPCION</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -17928,13 +17928,13 @@
         </is>
       </c>
       <c r="M269" s="2" t="n">
-        <v>2155.46</v>
+        <v>15787.98</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>2335-677-CM26</t>
+          <t>682-31-CM26</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -17954,22 +17954,22 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>69.130.301-2</t>
+          <t>61.802.014-2</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LINARES</t>
+          <t>MINISTERIO DE BIENES NACIONALES</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -17993,13 +17993,13 @@
         </is>
       </c>
       <c r="M270" s="2" t="n">
-        <v>107.93</v>
+        <v>2155.46</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>1515304-318-CM26</t>
+          <t>2335-677-CM26</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -18024,17 +18024,17 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>65.260.551-6</t>
+          <t>69.130.301-2</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>I MUNICIPALIDAD DE LINARES</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -18058,13 +18058,13 @@
         </is>
       </c>
       <c r="M271" s="2" t="n">
-        <v>9121.139999999999</v>
+        <v>107.93</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>1681-624-CM26</t>
+          <t>1515304-318-CM26</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -18084,22 +18084,22 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>61.606.917-9</t>
+          <t>65.260.551-6</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE LINARES</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -18123,13 +18123,13 @@
         </is>
       </c>
       <c r="M272" s="2" t="n">
-        <v>53236.72</v>
+        <v>9121.139999999999</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>1681-623-CM26</t>
+          <t>1681-624-CM26</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -18188,18 +18188,18 @@
         </is>
       </c>
       <c r="M273" s="2" t="n">
-        <v>39191.68</v>
+        <v>53236.72</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>4452-779-SE26</t>
+          <t>1681-623-CM26</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2239-13-LR23</t>
+          <t>2239-1-LR26</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -18219,12 +18219,12 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>61.606.903-9</t>
+          <t>61.606.917-9</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE CURICO</t>
+          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE LINARES</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
@@ -18253,18 +18253,18 @@
         </is>
       </c>
       <c r="M274" s="2" t="n">
-        <v>160327.63</v>
+        <v>39191.68</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>2410-443-CM26</t>
+          <t>4452-779-SE26</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2239-1-LR26</t>
+          <t>2239-13-LR23</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -18279,22 +18279,22 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>69.170.102-6</t>
+          <t>61.606.903-9</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LOS ANGELES</t>
+          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE CURICO</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -18318,13 +18318,13 @@
         </is>
       </c>
       <c r="M275" s="2" t="n">
-        <v>16737.44</v>
+        <v>160327.63</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>951405-316-CM26</t>
+          <t>2410-443-CM26</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -18344,22 +18344,22 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>61.980.840-1</t>
+          <t>69.170.102-6</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>I MUNICIPALIDAD DE LOS ANGELES</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18383,18 +18383,18 @@
         </is>
       </c>
       <c r="M276" s="2" t="n">
-        <v>2177.65</v>
+        <v>16737.44</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>1702-559-CM26</t>
+          <t>5052-637-SE26</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2239-1-LR26</t>
+          <t>2239-13-LR23</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -18404,7 +18404,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -18414,17 +18414,17 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>61.606.605-6</t>
+          <t>61.606.901-2</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD VINA DEL MAR QUILLOTA</t>
+          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE TALCA</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18448,13 +18448,13 @@
         </is>
       </c>
       <c r="M277" s="2" t="n">
-        <v>21615.78</v>
+        <v>274006.67</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>2045-298-CM26</t>
+          <t>951405-316-CM26</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -18469,7 +18469,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -18479,17 +18479,17 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>61.606.910-1</t>
+          <t>61.980.840-1</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE CUREPTO</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -18513,13 +18513,13 @@
         </is>
       </c>
       <c r="M278" s="2" t="n">
-        <v>8646.309999999999</v>
+        <v>2177.65</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>4469-814-CM26</t>
+          <t>1702-559-CM26</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -18539,17 +18539,17 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>70.754.700-6</t>
+          <t>61.606.605-6</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>UNIVERSIDAD DE PLAYA ANCHA DE CIENCIAS DE LA EDUCACION</t>
+          <t>SERVICIO DE SALUD VINA DEL MAR QUILLOTA</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
@@ -18578,13 +18578,13 @@
         </is>
       </c>
       <c r="M279" s="2" t="n">
-        <v>529.59</v>
+        <v>21615.78</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>2066-419-CM26</t>
+          <t>2045-298-CM26</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -18609,17 +18609,17 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>61.602.240-7</t>
+          <t>61.606.910-1</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Hospital Galvarino</t>
+          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE CUREPTO</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -18643,13 +18643,13 @@
         </is>
       </c>
       <c r="M280" s="2" t="n">
-        <v>12710.29</v>
+        <v>8646.309999999999</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>4469-815-CM26</t>
+          <t>4469-814-CM26</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -18708,13 +18708,13 @@
         </is>
       </c>
       <c r="M281" s="2" t="n">
-        <v>1482.84</v>
+        <v>529.59</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>1059253-2-CM26</t>
+          <t>2066-419-CM26</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -18739,17 +18739,17 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>69.073.100-2</t>
+          <t>61.602.240-7</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE SAN PEDRO</t>
+          <t>Hospital Galvarino</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -18773,13 +18773,13 @@
         </is>
       </c>
       <c r="M282" s="2" t="n">
-        <v>4431.23</v>
+        <v>12710.29</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>5067-2073-CM26</t>
+          <t>4469-815-CM26</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -18799,22 +18799,22 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>60.911.000-7</t>
+          <t>70.754.700-6</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>UNIVERSIDAD DE SANTIAGO DE CHILE</t>
+          <t>UNIVERSIDAD DE PLAYA ANCHA DE CIENCIAS DE LA EDUCACION</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -18838,13 +18838,13 @@
         </is>
       </c>
       <c r="M283" s="2" t="n">
-        <v>1080.79</v>
+        <v>1482.84</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>2145-809-CM26</t>
+          <t>1059253-2-CM26</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -18869,27 +18869,27 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>61.606.409-6</t>
+          <t>69.073.100-2</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL DE LOS VILOS</t>
+          <t>I MUNICIPALIDAD DE SAN PEDRO</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>Coquimbo</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -18903,13 +18903,13 @@
         </is>
       </c>
       <c r="M284" s="2" t="n">
-        <v>29721.7</v>
+        <v>4431.23</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>1057385-285-CM26</t>
+          <t>5067-2073-CM26</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -18934,17 +18934,17 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>61.606.204-2</t>
+          <t>60.911.000-7</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD ANTOFAGASTA HOSPITAL 21 DE MAYO TALTAL</t>
+          <t>UNIVERSIDAD DE SANTIAGO DE CHILE</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>Antofagasta</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -18968,13 +18968,13 @@
         </is>
       </c>
       <c r="M285" s="2" t="n">
-        <v>19594.7</v>
+        <v>1080.79</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>1320308-22-CM26</t>
+          <t>2145-809-CM26</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -18994,32 +18994,32 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>60.905.000-4</t>
+          <t>61.606.409-6</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
+          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL DE LOS VILOS</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -19033,13 +19033,13 @@
         </is>
       </c>
       <c r="M286" s="2" t="n">
-        <v>3810.6</v>
+        <v>29721.7</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>2125-1731-CM26</t>
+          <t>1057385-285-CM26</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -19064,27 +19064,27 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>61.606.407-k</t>
+          <t>61.606.204-2</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL DR. HUMBERTO ELORZA CORTES</t>
+          <t>SERVICIO DE SALUD ANTOFAGASTA HOSPITAL 21 DE MAYO TALTAL</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>Coquimbo</t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -19098,13 +19098,13 @@
         </is>
       </c>
       <c r="M287" s="2" t="n">
-        <v>77044.88</v>
+        <v>19594.7</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>2294-1704-CM26</t>
+          <t>1320308-22-CM26</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -19124,32 +19124,32 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>69.110.400-1</t>
+          <t>60.905.000-4</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE TALCA</t>
+          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -19163,13 +19163,13 @@
         </is>
       </c>
       <c r="M288" s="2" t="n">
-        <v>4064.2</v>
+        <v>3810.6</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>2147-397-CM26</t>
+          <t>2125-1731-CM26</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -19194,12 +19194,12 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>61.606.406-1</t>
+          <t>61.606.407-k</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL COMB</t>
+          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL DR. HUMBERTO ELORZA CORTES</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
@@ -19228,13 +19228,13 @@
         </is>
       </c>
       <c r="M289" s="2" t="n">
-        <v>13667.31</v>
+        <v>77044.88</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>1099402-452-CM26</t>
+          <t>2294-1704-CM26</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -19259,27 +19259,27 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>62.000.620-3</t>
+          <t>69.110.400-1</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>CENTRO DE SALUD FAMILIAR CESFAM LLAY LLAY</t>
+          <t>I MUNICIPALIDAD DE TALCA</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -19293,13 +19293,13 @@
         </is>
       </c>
       <c r="M290" s="2" t="n">
-        <v>12710.08</v>
+        <v>4064.2</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>2294-1703-CM26</t>
+          <t>2147-397-CM26</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -19324,27 +19324,27 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>69.110.400-1</t>
+          <t>61.606.406-1</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE TALCA</t>
+          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL COMB</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K291" t="inlineStr">
@@ -19358,13 +19358,13 @@
         </is>
       </c>
       <c r="M291" s="2" t="n">
-        <v>10494.76</v>
+        <v>13667.31</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>3951-227-CM26</t>
+          <t>1099402-452-CM26</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -19389,17 +19389,17 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>61.974.700-3</t>
+          <t>62.000.620-3</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>CONSULTORIO GENERAL URBANO VICTOR DOMINGO SILVA</t>
+          <t>CENTRO DE SALUD FAMILIAR CESFAM LLAY LLAY</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -19423,13 +19423,13 @@
         </is>
       </c>
       <c r="M292" s="2" t="n">
-        <v>10124.64</v>
+        <v>12710.08</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>1229788-202-CM26</t>
+          <t>2294-1703-CM26</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -19449,32 +19449,32 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>61.606.400-2</t>
+          <t>69.110.400-1</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD COQUIMBO</t>
+          <t>I MUNICIPALIDAD DE TALCA</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>Coquimbo</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K293" t="inlineStr">
@@ -19488,13 +19488,13 @@
         </is>
       </c>
       <c r="M293" s="2" t="n">
-        <v>25827.57</v>
+        <v>10494.76</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>1978-952-CM26</t>
+          <t>3951-227-CM26</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -19514,22 +19514,22 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>61.606.900-4</t>
+          <t>61.974.700-3</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL MAULE</t>
+          <t>CONSULTORIO GENERAL URBANO VICTOR DOMINGO SILVA</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -19553,13 +19553,13 @@
         </is>
       </c>
       <c r="M294" s="2" t="n">
-        <v>42366.93</v>
+        <v>10124.64</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>3849-26-CM26</t>
+          <t>1229788-202-CM26</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -19579,32 +19579,32 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>60.505.000-K</t>
+          <t>61.606.400-2</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SERVICIO DE SALUD COQUIMBO</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -19618,13 +19618,13 @@
         </is>
       </c>
       <c r="M295" s="2" t="n">
-        <v>1975.36</v>
+        <v>25827.57</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>1529-230-CM26</t>
+          <t>1978-952-CM26</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -19644,32 +19644,32 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>61.602.140-0</t>
+          <t>61.606.900-4</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD HOSPITAL DE RENGO</t>
+          <t>SERVICIO DE SALUD DEL MAULE</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -19683,13 +19683,13 @@
         </is>
       </c>
       <c r="M296" s="2" t="n">
-        <v>51773.38</v>
+        <v>42366.93</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>507428-892-CM26</t>
+          <t>3849-26-CM26</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -19714,17 +19714,17 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>61.979.210-6</t>
+          <t>60.505.000-K</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD CHILOE</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>Los Lagos</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -19748,13 +19748,13 @@
         </is>
       </c>
       <c r="M297" s="2" t="n">
-        <v>31775.2</v>
+        <v>1975.36</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>3787-49-CM26</t>
+          <t>1529-230-CM26</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -19774,32 +19774,32 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>60.505.000-K</t>
+          <t>61.602.140-0</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SERVICIO DE SALUD HOSPITAL DE RENGO</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -19813,13 +19813,13 @@
         </is>
       </c>
       <c r="M298" s="2" t="n">
-        <v>10873.47</v>
+        <v>51773.38</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>1426099-177-CM26</t>
+          <t>507428-892-CM26</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -19839,22 +19839,22 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>62.000.970-9</t>
+          <t>61.979.210-6</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>SERVICIO NACIONAL DE REINSERCION SOCIAL JUVENIL</t>
+          <t>SERVICIO DE SALUD CHILOE</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -19878,13 +19878,13 @@
         </is>
       </c>
       <c r="M299" s="2" t="n">
-        <v>2647.93</v>
+        <v>31775.2</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>1395-688-CM26</t>
+          <t>3787-49-CM26</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -19904,32 +19904,32 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>61.606.400-2</t>
+          <t>60.505.000-K</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD COQUIMBO</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>Coquimbo</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -19943,13 +19943,13 @@
         </is>
       </c>
       <c r="M300" s="2" t="n">
-        <v>40696.68</v>
+        <v>10873.47</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>4696-9-CM26</t>
+          <t>1426099-177-CM26</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -19964,7 +19964,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -19974,27 +19974,27 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>60.901.000-2</t>
+          <t>62.000.970-9</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
+          <t>SERVICIO NACIONAL DE REINSERCION SOCIAL JUVENIL</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -20008,13 +20008,13 @@
         </is>
       </c>
       <c r="M301" s="2" t="n">
-        <v>1476.94</v>
+        <v>2647.93</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>1464-1326-CM26</t>
+          <t>1395-688-CM26</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -20029,7 +20029,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -20039,27 +20039,27 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>61.606.918-7</t>
+          <t>61.606.400-2</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE PARRAL</t>
+          <t>SERVICIO DE SALUD COQUIMBO</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -20073,13 +20073,13 @@
         </is>
       </c>
       <c r="M302" s="2" t="n">
-        <v>37652.55</v>
+        <v>40696.68</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>4232-76-CM26</t>
+          <t>4696-9-CM26</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -20099,32 +20099,32 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>60.505.101-4</t>
+          <t>60.901.000-2</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
         </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>Arica y Parinacota</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J303" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K303" t="inlineStr">
@@ -20138,13 +20138,13 @@
         </is>
       </c>
       <c r="M303" s="2" t="n">
-        <v>22705.44</v>
+        <v>1476.94</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>1057440-470-CM26</t>
+          <t>1464-1326-CM26</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -20164,22 +20164,22 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>61.606.403-7</t>
+          <t>61.606.918-7</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL DE COQUIMBO</t>
+          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE PARRAL</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>Coquimbo</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -20203,13 +20203,13 @@
         </is>
       </c>
       <c r="M304" s="2" t="n">
-        <v>8725.440000000001</v>
+        <v>37652.55</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>1057390-658-CM26</t>
+          <t>4232-76-CM26</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -20234,17 +20234,17 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>61.955.100-1</t>
+          <t>60.505.101-4</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD ARAUCANIA NORTE</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Arica y Parinacota</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -20268,13 +20268,13 @@
         </is>
       </c>
       <c r="M305" s="2" t="n">
-        <v>10546.93</v>
+        <v>22705.44</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2085-736-CM26</t>
+          <t>1057440-470-CM26</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -20299,17 +20299,17 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>61.602.226-1</t>
+          <t>61.606.403-7</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD ARAUCANIA HOSPITAL DE TRAIGUEN</t>
+          <t>SERVICIO DE SALUD COQUIMBO HOSPITAL DE COQUIMBO</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -20333,13 +20333,13 @@
         </is>
       </c>
       <c r="M306" s="2" t="n">
-        <v>28639.57</v>
+        <v>8725.440000000001</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>5349-1763-CM26</t>
+          <t>1057390-658-CM26</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -20364,17 +20364,17 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>61.606.303-0</t>
+          <t>61.955.100-1</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>HOSPITAL PROVINCIAL   DEL HUASCO MSR FERNANDO ARIZTIA RUIZ</t>
+          <t>SERVICIO DE SALUD ARAUCANIA NORTE</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>Atacama</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -20398,13 +20398,13 @@
         </is>
       </c>
       <c r="M307" s="2" t="n">
-        <v>60473.35</v>
+        <v>10546.93</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>4696-10-CM26</t>
+          <t>2085-736-CM26</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -20429,27 +20429,27 @@
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>60.901.000-2</t>
+          <t>61.602.226-1</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
+          <t>SERVICIO DE SALUD ARAUCANIA HOSPITAL DE TRAIGUEN</t>
         </is>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J308" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -20463,13 +20463,13 @@
         </is>
       </c>
       <c r="M308" s="2" t="n">
-        <v>564.54</v>
+        <v>28639.57</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>1978-957-CM26</t>
+          <t>5349-1763-CM26</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -20489,22 +20489,22 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>61.606.900-4</t>
+          <t>61.606.303-0</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL MAULE</t>
+          <t>HOSPITAL PROVINCIAL   DEL HUASCO MSR FERNANDO ARIZTIA RUIZ</t>
         </is>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -20528,13 +20528,13 @@
         </is>
       </c>
       <c r="M309" s="2" t="n">
-        <v>630.66</v>
+        <v>60473.35</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>778989-161-CM26</t>
+          <t>4696-10-CM26</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -20554,32 +20554,32 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>65.081.190-9</t>
+          <t>60.901.000-2</t>
         </is>
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
         </is>
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>Antofagasta</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
@@ -20593,13 +20593,13 @@
         </is>
       </c>
       <c r="M310" s="2" t="n">
-        <v>430.49</v>
+        <v>564.54</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>1099899-138-CM26</t>
+          <t>1978-957-CM26</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -20619,22 +20619,22 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>62.000.630-0</t>
+          <t>61.606.900-4</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>CENTRO SALUD MENTAL COMUNITARIA LOS ANDES</t>
+          <t>SERVICIO DE SALUD DEL MAULE</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
@@ -20658,13 +20658,13 @@
         </is>
       </c>
       <c r="M311" s="2" t="n">
-        <v>7454.57</v>
+        <v>630.66</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>1099899-137-CM26</t>
+          <t>778989-161-CM26</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -20689,17 +20689,17 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>62.000.630-0</t>
+          <t>65.081.190-9</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>CENTRO SALUD MENTAL COMUNITARIA LOS ANDES</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -20723,13 +20723,13 @@
         </is>
       </c>
       <c r="M312" s="2" t="n">
-        <v>1412.76</v>
+        <v>430.49</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>585-111-CM26</t>
+          <t>1099899-138-CM26</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -20749,22 +20749,22 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>82.174.900-k</t>
+          <t>62.000.630-0</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>SERVICIO DE COOPERACION TECNICA</t>
+          <t>CENTRO SALUD MENTAL COMUNITARIA LOS ANDES</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -20788,13 +20788,13 @@
         </is>
       </c>
       <c r="M313" s="2" t="n">
-        <v>289.72</v>
+        <v>7454.57</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>545598-752-CM26</t>
+          <t>1099899-137-CM26</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -20814,22 +20814,22 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>71.149.700-5</t>
+          <t>62.000.630-0</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>CORP MUNICIPAL DE CASTRO PARA LA EDUCACION SALUD Y ATENCION AL MENOR</t>
+          <t>CENTRO SALUD MENTAL COMUNITARIA LOS ANDES</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>Los Lagos</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -20853,13 +20853,13 @@
         </is>
       </c>
       <c r="M314" s="2" t="n">
-        <v>4394.59</v>
+        <v>1412.76</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>3950-1348-CM26</t>
+          <t>585-111-CM26</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -20879,22 +20879,22 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>61.974.600-7</t>
+          <t>82.174.900-k</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>DIRECCION SALUD RURAL</t>
+          <t>SERVICIO DE COOPERACION TECNICA</t>
         </is>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -20918,13 +20918,13 @@
         </is>
       </c>
       <c r="M315" s="2" t="n">
-        <v>6419.39</v>
+        <v>289.72</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>1079566-332-CM26</t>
+          <t>545598-752-CM26</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -20944,32 +20944,32 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>61.979.370-6</t>
+          <t>71.149.700-5</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>CORP MUNICIPAL DE CASTRO PARA LA EDUCACION SALUD Y ATENCION AL MENOR</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J316" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
@@ -20983,13 +20983,13 @@
         </is>
       </c>
       <c r="M316" s="2" t="n">
-        <v>521758.93</v>
+        <v>4394.59</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>4605-94-CM26</t>
+          <t>3950-1348-CM26</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -21014,17 +21014,17 @@
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>61.819.000-5</t>
+          <t>61.974.600-7</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>SERVICIO DE VIVIENDA Y URBANIZACION VII REGION</t>
+          <t>DIRECCION SALUD RURAL</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -21048,13 +21048,13 @@
         </is>
       </c>
       <c r="M317" s="2" t="n">
-        <v>2438.44</v>
+        <v>6419.39</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>1057379-444-CM26</t>
+          <t>1079566-332-CM26</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -21079,27 +21079,27 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>61.606.703-6</t>
+          <t>61.979.370-6</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD ACONCAGUA HOSPITAL DE PUTAENDO</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -21113,13 +21113,13 @@
         </is>
       </c>
       <c r="M318" s="2" t="n">
-        <v>3270.39</v>
+        <v>521758.93</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>4696-8-CM26</t>
+          <t>4605-94-CM26</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -21139,32 +21139,32 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>60.901.000-2</t>
+          <t>61.819.000-5</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
+          <t>SERVICIO DE VIVIENDA Y URBANIZACION VII REGION</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J319" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -21178,71 +21178,201 @@
         </is>
       </c>
       <c r="M319" s="2" t="n">
-        <v>402.12</v>
+        <v>2438.44</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
+          <t>1057379-444-CM26</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>2239-1-LR26</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>ago-2026</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Recepcion Conforme</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>61.606.703-6</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>SERVICIO DE SALUD ACONCAGUA HOSPITAL DE PUTAENDO</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Valparaíso</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>96.781.350-8</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M320" s="2" t="n">
+        <v>3270.39</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>4696-8-CM26</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>2239-1-LR26</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>ago-2026</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Aceptada</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>60.901.000-2</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>96.556.930-8</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M321" s="2" t="n">
+        <v>402.12</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
           <t>1271178-294-CM26</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>2239-1-LR26</t>
-        </is>
-      </c>
-      <c r="C320" t="inlineStr">
-        <is>
-          <t>ago-2026</t>
-        </is>
-      </c>
-      <c r="D320" t="inlineStr">
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>2239-1-LR26</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>ago-2026</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E320" t="inlineStr">
-        <is>
-          <t>Recepcion Conforme</t>
-        </is>
-      </c>
-      <c r="F320" t="inlineStr">
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Recepcion Conforme</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
         <is>
           <t>71.369.900-4</t>
         </is>
       </c>
-      <c r="G320" t="inlineStr">
+      <c r="G322" t="inlineStr">
         <is>
           <t>CORPORACION MUNICIPAL DE DESARROLLO SOCIAL DE MACUL</t>
         </is>
       </c>
-      <c r="H320" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
-      <c r="I320" t="inlineStr">
-        <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
-        </is>
-      </c>
-      <c r="J320" t="inlineStr">
-        <is>
-          <t>96.781.350-8</t>
-        </is>
-      </c>
-      <c r="K320" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
-      <c r="L320" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="M320" s="2" t="n">
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>96.781.350-8</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M322" s="2" t="n">
         <v>8788.860000000001</v>
       </c>
     </row>

</xml_diff>